<commit_message>
Daily EOD data and reports for 2026-07-31
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260731.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260731.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.36</v>
+        <v>1.362</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.045</v>
+        <v>0.047</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>208326.16</v>
+        <v>208632.52</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>6893.15</v>
+        <v>7199.51</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.185</v>
+        <v>2.175</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.035</v>
+        <v>0.025</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>152950</v>
+        <v>152250</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2450</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.005</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.06</v>
+        <v>0.055</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>5.82%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>57745.29</v>
+        <v>57458</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3447.48</v>
+        <v>3160.19</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60.745</v>
+        <v>60.8</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1.595</v>
+        <v>1.65</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.70%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>672143.42</v>
+        <v>672752</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>17648.67</v>
+        <v>18257.25</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>178.61</v>
+        <v>178.67</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>124.17</v>
+        <v>122.66</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-3.76</v>
+        <v>-5.27</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-4.12%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>496680</v>
+        <v>490640</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-15040</v>
+        <v>-21080</v>
       </c>
     </row>
     <row r="12">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.26</v>
+        <v>33.255</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.36</v>
+        <v>0.355</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42838.88</v>
+        <v>42832.44</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>463.68</v>
+        <v>457.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1644658.4</v>
+        <v>1638539.6</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>14682.98</v>
+        <v>8564.190000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>